<commit_message>
Raise Units 1-5 MCQ banks to benchmark quality
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Python/Unit 3 - Control Flow/Unit 3 - Control Flow - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Python/Unit 3 - Control Flow/Unit 3 - Control Flow - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 3" sheetId="1" r:id="Rb417f061462647a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 3" sheetId="1" r:id="R62edd5e623334167"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -502,16 +502,16 @@
         <x:v>No ID entered — the text "0" counts as empty</x:v>
       </x:c>
       <x:c r="N2" t="str">
+        <x:v>Tracking parcel — "0" has one character, so it is not empty</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
         <x:v>An error — you cannot put a string after if</x:v>
-      </x:c>
-      <x:c r="O2" t="str">
-        <x:v>Tracking parcel — "0" has one character, so it is not empty</x:v>
       </x:c>
       <x:c r="P2" t="str">
         <x:v>No ID entered — Python turns "0" into the number 0 first</x:v>
       </x:c>
       <x:c r="Q2" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="18" customHeight="1">
@@ -622,16 +622,16 @@
         <x:v>Because 95 is not greater than 90</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>Because the first true condition wins — marks &gt;= 60 matches first, so the rest are skipped</x:v>
+        <x:v>Because an elif chain prints every branch that is true</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>Because an elif chain prints every branch that is true</x:v>
+        <x:v>Because the else branch is missing</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>Because the else branch is missing</x:v>
+        <x:v>Because the first true condition wins</x:v>
       </x:c>
       <x:c r="Q4" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -681,16 +681,16 @@
         <x:v>&gt; should be !=; it shows No discount</x:v>
       </x:c>
       <x:c r="N5" t="str">
+        <x:v>&gt; should be &gt;=; it shows No discount</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
         <x:v>There is no bug; it shows Discount applied</x:v>
-      </x:c>
-      <x:c r="O5" t="str">
-        <x:v>&gt; should be &gt;=; it shows No discount</x:v>
       </x:c>
       <x:c r="P5" t="str">
         <x:v>&gt; should be ==; it shows Discount applied</x:v>
       </x:c>
       <x:c r="Q5" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -739,19 +739,19 @@
       </x:c>
       <x:c r="L6"/>
       <x:c r="M6" t="str">
-        <x:v>Gold — only the top badge shows</x:v>
+        <x:v>Gold</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>Bronze — the first true line stops the rest</x:v>
+        <x:v>Bronze</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>Nothing — the ranges clash</x:v>
+        <x:v>Bronze, Silver, and Gold</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>Bronze, Silver, and Gold — each if runs on its own</x:v>
+        <x:v>Nothing</x:v>
       </x:c>
       <x:c r="Q6" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -916,13 +916,13 @@
         <x:v>No — Version B skips the soil check</x:v>
       </x:c>
       <x:c r="O9" t="str">
+        <x:v>Yes — both water only when the soil is dry and the tank has water</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
         <x:v>No — Version A checks the tank even when the soil is wet</x:v>
       </x:c>
-      <x:c r="P9" t="str">
-        <x:v>Yes — both water only when the soil is dry and the tank has water</x:v>
-      </x:c>
       <x:c r="Q9" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -930,27 +930,18 @@
         <x:v>Python - MCQ - 3.1.9</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>A site accepts a coupon only if it is 8 characters long and not already used. Two coders write the check, then test a 5-character coupon that has never been used:
-```python
-used = False
-code = input("Enter coupon: ")
-# Option 1
-if len(code) != 8:
-    print("Wrong length")
-elif used:
-    print("Already used")
+        <x:v>A signup form intends to reject non-numeric ages before comparing them, but the checks are in an unsafe order:
+```python
+entry = input("Age: ")
+if int(entry) &lt; 18 or not entry.isdigit():
+    print("Invalid age")
 else:
-    print("Coupon applied")
-# Option 2
-if len(code) != 8 and used:
-    print("Invalid coupon")
-else:
-    print("Coupon applied")
-```
-Which version rejects the bad coupon, and why does the other let it through?</x:v>
+    print("Accepted")
+```
+Which input exposes the ordering defect by crashing before the validation message can run?</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Option 1 checks the two rules one after another, so the wrong length is caught. Option 2 joins them with `and`, so it only rejects a coupon that is BOTH the wrong length AND already used. A 5-character unused coupon fails only one rule, so Option 2 prints `Coupon applied` and lets it through.</x:v>
+        <x:v>With `"x"`, Python tries `int("x")` first and raises `ValueError`; it never reaches `.isdigit()`. Numeric text such as `"17"`, `"25"`, or `"0"` converts successfully. The safe order checks `not entry.isdigit()` before any conversion.</x:v>
       </x:c>
       <x:c r="D10" t="n">
         <x:v>10</x:v>
@@ -978,16 +969,16 @@
       </x:c>
       <x:c r="L10"/>
       <x:c r="M10" t="str">
-        <x:v>Option 1 rejects it; Option 2 only rejects a coupon that is the wrong length AND already used</x:v>
+        <x:v>`x`</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>Both reject it; the two versions behave the same</x:v>
+        <x:v>`17`</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>Option 2 rejects it; Option 1 just adds extra branches for no reason</x:v>
+        <x:v>`25`</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>Option 1 rejects it; Option 2 fails because only one of the two checks matters</x:v>
+        <x:v>`0`</x:v>
       </x:c>
       <x:c r="Q10" t="n">
         <x:v>1</x:v>
@@ -1041,13 +1032,13 @@
         <x:v>"Light" if weight &gt; 3000 else "Heavy"</x:v>
       </x:c>
       <x:c r="O11" t="str">
+        <x:v>"Heavy" if weight &gt; 3000</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
         <x:v>"Heavy" if weight &gt; 3000 else "Light"</x:v>
       </x:c>
-      <x:c r="P11" t="str">
-        <x:v>"Heavy" if weight &gt; 3000</x:v>
-      </x:c>
       <x:c r="Q11" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1055,15 +1046,18 @@
         <x:v>Python - MCQ - 3.2.1</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>A ward monitor should alert when the temperature reaches 38.0°C. A tester wants the single reading that would reveal the bug if someone wrote `&gt;` instead of `&gt;=`:
-```python
-def needs_alert(temp):
-    return temp &gt;= 38.0
-```
-Which reading must be in the test?</x:v>
+        <x:v>A ward monitor should alert when the temperature reaches 38.0°C, but its comparison excludes the exact boundary:
+```python
+temp = 38.0
+if temp &gt; 38.0:
+    print("Alert")
+else:
+    print("Normal")
+```
+Which test reading exposes the boundary defect?</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>`&gt;=` and `&gt;` give different answers only at the exact number. `needs_alert(38.0)` is True with `&gt;=`, but would be False with `&gt;`. Any reading away from 38.0 gives the same answer either way, so only 38.0 catches the mistake.</x:v>
+        <x:v>The incorrect `&gt;` and the required `&gt;=` differ only at exactly 38.0. At that reading, the current code prints `Normal`, while the rule requires `Alert`. Values above or below the boundary do not distinguish the two operators.</x:v>
       </x:c>
       <x:c r="D12" t="n">
         <x:v>8</x:v>
@@ -1172,15 +1166,18 @@
         <x:v>Python - MCQ - 3.2.3</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>During testing, this age check is always called with whole numbers, and every call passes. But in the real app the value comes straight from `input()`:
-```python
-def check_can_vote(age):
-    return "Eligible" if age &gt;= 18 else "Not eligible"
-```
-Which single call behaves like the real app and reveals the hidden problem?</x:v>
+        <x:v>An age arrives directly from `input()`, so it is text when the comparison runs:
+```python
+age = input("Age: ")
+if age &gt;= 18:
+    print("Eligible")
+else:
+    print("Not eligible")
+```
+Which is the smallest correct repair?</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>`input()` always returns a string, so the real app passes text like `"25"`. Comparing `"25" &gt;= 18` compares a string to a number, which raises a `TypeError` in Python 3. Calls with plain numbers — normal or extreme — never hit this, which is why the tests missed it.</x:v>
+        <x:v>`input()` returns text, and text cannot be ordered against the integer 18. Converting at the point of input with `age = int(input("Age: "))` makes both sides numeric before the comparison. Comparing with the text `"18"` would use character ordering rather than numeric age ordering.</x:v>
       </x:c>
       <x:c r="D14" t="n">
         <x:v>8</x:v>
@@ -1208,19 +1205,19 @@
       </x:c>
       <x:c r="L14"/>
       <x:c r="M14" t="str">
-        <x:v>check_can_vote("25")</x:v>
+        <x:v>Use `age = str(input("Age: "))`</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>check_can_vote(25)</x:v>
+        <x:v>Use `age = input("Age: ") + 0`</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>check_can_vote(16)</x:v>
+        <x:v>Use `age = int(input("Age: "))`</x:v>
       </x:c>
       <x:c r="P14" t="str">
-        <x:v>check_can_vote(0)</x:v>
+        <x:v>Change the test to `age &gt;= "18"`</x:v>
       </x:c>
       <x:c r="Q14" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1270,16 +1267,16 @@
         <x:v>It should be &gt;= 14 to include the 14th day</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>Nothing is wrong — 20 days is within the limit</x:v>
+        <x:v>&lt; should be &gt;</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>&lt; should be &gt; — the fee is for more than 14 days, not fewer</x:v>
+        <x:v>Nothing is wrong</x:v>
       </x:c>
       <x:c r="P15" t="str">
         <x:v>The else branch should print the fee</x:v>
       </x:c>
       <x:c r="Q15" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1329,7 +1326,7 @@
         <x:v>The comparisons are backwards</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>and should be or — no number is below -50 and above 150 at once</x:v>
+        <x:v>and should be or</x:v>
       </x:c>
       <x:c r="O16" t="str">
         <x:v>The else needs its own condition</x:v>
@@ -1513,13 +1510,13 @@
         <x:v>active and checked_in</x:v>
       </x:c>
       <x:c r="O19" t="str">
+        <x:v>not active and not checked_in</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
         <x:v>active and not checked_in</x:v>
       </x:c>
-      <x:c r="P19" t="str">
-        <x:v>not active and not checked_in</x:v>
-      </x:c>
       <x:c r="Q19" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1568,10 +1565,10 @@
       </x:c>
       <x:c r="L20"/>
       <x:c r="M20" t="str">
+        <x:v>Version A stores "Approved", Version B stores "Rejected"</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
         <x:v>Both store "Approved"</x:v>
-      </x:c>
-      <x:c r="N20" t="str">
-        <x:v>Version A stores "Approved", Version B stores "Rejected"</x:v>
       </x:c>
       <x:c r="O20" t="str">
         <x:v>Both store "Rejected"</x:v>
@@ -1580,7 +1577,7 @@
         <x:v>Version A stores "Rejected", Version B stores "Approved"</x:v>
       </x:c>
       <x:c r="Q20" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1650,11 +1647,10 @@
         <x:v>Python - MCQ - 3.2.11</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>A dashboard shows one label per rating: under 3 is "Improve", 3 to 4 is "Meets", over 4 is "Exceeds". It must never show two labels, and never show none.
-Which structure guarantees exactly one label for any rating?</x:v>
+        <x:v>A dashboard has mutually exclusive rating bands and needs a clear fallback for any value not covered explicitly. Which structure communicates that design most directly?</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>An `if`-`elif`-`else` chain runs only the first matching branch, and the `else` covers everything left over — so exactly one label always shows. Separate `if`s could fire more than once, one `if` with `or` cannot pick a different label per range, and `match-case` is for fixed values, not ranges.</x:v>
+        <x:v>An `if`-`elif`-`else` chain makes the mutual exclusivity explicit: the first matching band runs and the final `else` provides a fallback. Carefully written separate `if` statements could also be mutually exclusive, but the chain expresses the intended one-path design more clearly and is safer to maintain.</x:v>
       </x:c>
       <x:c r="D22" t="n">
         <x:v>8</x:v>
@@ -1682,16 +1678,16 @@
       </x:c>
       <x:c r="L22"/>
       <x:c r="M22" t="str">
-        <x:v>An if-elif-else chain</x:v>
+        <x:v>An `if`-`elif`-`else` chain</x:v>
       </x:c>
       <x:c r="N22" t="str">
-        <x:v>Three separate if statements</x:v>
+        <x:v>Three unrelated `if` statements</x:v>
       </x:c>
       <x:c r="O22" t="str">
-        <x:v>One if with the ranges joined by or</x:v>
+        <x:v>One `if` joining every band with `or`</x:v>
       </x:c>
       <x:c r="P22" t="str">
-        <x:v>A match-case that compares the rating to each number</x:v>
+        <x:v>A `match` comparing every possible rating</x:v>
       </x:c>
       <x:c r="Q22" t="n">
         <x:v>1</x:v>
@@ -1744,19 +1740,19 @@
       </x:c>
       <x:c r="L23"/>
       <x:c r="M23" t="str">
+        <x:v>The order is wrong</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
         <x:v>The else should say gb &gt; 10</x:v>
       </x:c>
-      <x:c r="N23" t="str">
+      <x:c r="O23" t="str">
         <x:v>Every &lt;= should be &lt;</x:v>
-      </x:c>
-      <x:c r="O23" t="str">
-        <x:v>The order is wrong — gb &lt;= 10 catches small usage first</x:v>
       </x:c>
       <x:c r="P23" t="str">
         <x:v>The free and top tiers need a lower bound with and</x:v>
       </x:c>
       <x:c r="Q23" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1808,16 +1804,16 @@
         <x:v>Invalid card</x:v>
       </x:c>
       <x:c r="N24" t="str">
+        <x:v>Unlocked</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
         <x:v>Nothing</x:v>
-      </x:c>
-      <x:c r="O24" t="str">
-        <x:v>Unlocked</x:v>
       </x:c>
       <x:c r="P24" t="str">
         <x:v>Both Unlocked and Invalid card</x:v>
       </x:c>
       <x:c r="Q24" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1872,16 +1868,16 @@
         <x:v>English selected — match ignores capitals</x:v>
       </x:c>
       <x:c r="N25" t="str">
+        <x:v>Language not supported — "EN" does not equal "en", so no case matches</x:v>
+      </x:c>
+      <x:c r="O25" t="str">
         <x:v>Nothing — match errors when no case matches</x:v>
       </x:c>
-      <x:c r="O25" t="str">
+      <x:c r="P25" t="str">
         <x:v>English selected — the _ case jumps to the first case</x:v>
       </x:c>
-      <x:c r="P25" t="str">
-        <x:v>Language not supported — "EN" does not equal "en", so no case matches</x:v>
-      </x:c>
       <x:c r="Q25" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1928,10 +1924,10 @@
       </x:c>
       <x:c r="L26"/>
       <x:c r="M26" t="str">
+        <x:v>Subject required — a string of only spaces counts as empty</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
         <x:v>Ticket created — spaces still count as characters, so the string is not empty</x:v>
-      </x:c>
-      <x:c r="N26" t="str">
-        <x:v>Subject required — a string of only spaces counts as empty</x:v>
       </x:c>
       <x:c r="O26" t="str">
         <x:v>An error — spaces cannot be tested in an if</x:v>
@@ -1940,7 +1936,7 @@
         <x:v>Subject required — Python removes the spaces first</x:v>
       </x:c>
       <x:c r="Q26" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1996,16 +1992,16 @@
         <x:v>Robot idle</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>Order queued — waiting for a slot</x:v>
+        <x:v>Idle move to zone</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>Idle move to zone</x:v>
+        <x:v>Order queued</x:v>
       </x:c>
       <x:c r="P27" t="str">
         <x:v>Robot dispatched</x:v>
       </x:c>
       <x:c r="Q27" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2113,16 +2109,16 @@
         <x:v>systolic &gt; 90 and systolic &lt; 120</x:v>
       </x:c>
       <x:c r="N29" t="str">
+        <x:v>90 &lt;= systolic &lt;= 120</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
         <x:v>systolic &gt;= 90 or systolic &lt;= 120</x:v>
       </x:c>
-      <x:c r="O29" t="str">
+      <x:c r="P29" t="str">
         <x:v>systolic == 90 and systolic == 120</x:v>
       </x:c>
-      <x:c r="P29" t="str">
-        <x:v>90 &lt;= systolic &lt;= 120</x:v>
-      </x:c>
       <x:c r="Q29" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2171,19 +2167,19 @@
       </x:c>
       <x:c r="L30"/>
       <x:c r="M30" t="str">
-        <x:v>The second branch — it repeats the first condition; the customer sees Free next-day delivery</x:v>
+        <x:v>The else</x:v>
       </x:c>
       <x:c r="N30" t="str">
-        <x:v>The else — the customer sees Free standard delivery</x:v>
+        <x:v>The if and the elif both</x:v>
       </x:c>
       <x:c r="O30" t="str">
-        <x:v>The if and the elif both — everyone sees Paid delivery</x:v>
+        <x:v>The second branch</x:v>
       </x:c>
       <x:c r="P30" t="str">
-        <x:v>None — all three run and two lines print</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="Q30" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2231,16 +2227,16 @@
         <x:v>"Qualified" if score &gt; 60 else "Try again"</x:v>
       </x:c>
       <x:c r="N31" t="str">
+        <x:v>if score &gt;= 60: "Qualified" else: "Try again"</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>"Try again" if score &gt;= 60 else "Qualified"</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
         <x:v>"Qualified" if score &gt;= 60 else "Try again"</x:v>
       </x:c>
-      <x:c r="O31" t="str">
-        <x:v>if score &gt;= 60: "Qualified" else: "Try again"</x:v>
-      </x:c>
-      <x:c r="P31" t="str">
-        <x:v>"Try again" if score &gt;= 60 else "Qualified"</x:v>
-      </x:c>
       <x:c r="Q31" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2285,19 +2281,19 @@
       </x:c>
       <x:c r="L32"/>
       <x:c r="M32" t="str">
+        <x:v>stock &lt; 20</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
         <x:v>stock &lt;= 20</x:v>
       </x:c>
-      <x:c r="N32" t="str">
+      <x:c r="O32" t="str">
         <x:v>stock &gt; 20</x:v>
-      </x:c>
-      <x:c r="O32" t="str">
-        <x:v>stock &lt; 20</x:v>
       </x:c>
       <x:c r="P32" t="str">
         <x:v>stock == 20</x:v>
       </x:c>
       <x:c r="Q32" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2355,13 +2351,13 @@
         <x:v>Yes — they differ at temp == 17</x:v>
       </x:c>
       <x:c r="O33" t="str">
+        <x:v>No — one of the two opposite conditions is always true, so both set the same value</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
         <x:v>Yes — two ifs always set the value twice</x:v>
       </x:c>
-      <x:c r="P33" t="str">
-        <x:v>No — one of the two opposite conditions is always true, so both set the same value</x:v>
-      </x:c>
       <x:c r="Q33" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2414,19 +2410,19 @@
       </x:c>
       <x:c r="L34"/>
       <x:c r="M34" t="str">
+        <x:v>Yes — they always match</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>No — Version A flags small foreign payments</x:v>
+      </x:c>
+      <x:c r="O34" t="str">
         <x:v>No — Version A prints nothing, but Version B prints Domestic large payment</x:v>
-      </x:c>
-      <x:c r="N34" t="str">
-        <x:v>Yes — they always match</x:v>
-      </x:c>
-      <x:c r="O34" t="str">
-        <x:v>No — Version A flags small foreign payments</x:v>
       </x:c>
       <x:c r="P34" t="str">
         <x:v>No — Version B never checks foreign</x:v>
       </x:c>
       <x:c r="Q34" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2482,16 +2478,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N35" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="P35" t="str">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O35" t="str">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="P35" t="str">
-        <x:v>100</x:v>
-      </x:c>
       <x:c r="Q35" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2538,19 +2534,19 @@
       </x:c>
       <x:c r="L36"/>
       <x:c r="M36" t="str">
-        <x:v>Prints Processing 50 — isdigit ignores the letter</x:v>
+        <x:v>Prints Processing 50</x:v>
       </x:c>
       <x:c r="N36" t="str">
         <x:v>Crashes on int() with an error</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>Prints Enter numbers only — "50x" is not all digits</x:v>
+        <x:v>Prints Processing 50x</x:v>
       </x:c>
       <x:c r="P36" t="str">
-        <x:v>Prints Processing 50x</x:v>
+        <x:v>Prints Enter numbers only</x:v>
       </x:c>
       <x:c r="Q36" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2600,19 +2596,19 @@
       </x:c>
       <x:c r="L37"/>
       <x:c r="M37" t="str">
-        <x:v>Nothing stops it — Upload accepted</x:v>
+        <x:v>Nothing stops it</x:v>
       </x:c>
       <x:c r="N37" t="str">
-        <x:v>The name check stops it — File name required</x:v>
+        <x:v>The name check stops it</x:v>
       </x:c>
       <x:c r="O37" t="str">
+        <x:v>The size check stops it</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
         <x:v>It crashes comparing size to 5</x:v>
       </x:c>
-      <x:c r="P37" t="str">
-        <x:v>The size check stops it — File too large</x:v>
-      </x:c>
       <x:c r="Q37" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2661,10 +2657,10 @@
       </x:c>
       <x:c r="L38"/>
       <x:c r="M38" t="str">
+        <x:v>Menu closed only</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
         <x:v>Balance, then Menu closed</x:v>
-      </x:c>
-      <x:c r="N38" t="str">
-        <x:v>Menu closed only</x:v>
       </x:c>
       <x:c r="O38" t="str">
         <x:v>An error because case _ is required</x:v>
@@ -2673,7 +2669,7 @@
         <x:v>Nothing</x:v>
       </x:c>
       <x:c r="Q38" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2794,14 +2790,14 @@
 `else: print("Must be 18 or older")`</x:v>
       </x:c>
       <x:c r="N40" t="str">
+        <x:v>`if not entry.isdigit(): print("Digits only")`
+`elif int(entry) &lt; 18: print("Must be 18 or older")`
+`else: print("Accepted")`</x:v>
+      </x:c>
+      <x:c r="O40" t="str">
         <x:v>`if entry.isdigit(): print("Accepted")`
 `elif int(entry) &lt; 18: print("Must be 18 or older")`
 `else: print("Digits only")`</x:v>
-      </x:c>
-      <x:c r="O40" t="str">
-        <x:v>`if not entry.isdigit(): print("Digits only")`
-`elif int(entry) &lt; 18: print("Must be 18 or older")`
-`else: print("Accepted")`</x:v>
       </x:c>
       <x:c r="P40" t="str">
         <x:v>`if not entry.isdigit(): print("Digits only")`
@@ -2809,7 +2805,7 @@
 `else: print("Accepted")`</x:v>
       </x:c>
       <x:c r="Q40" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="41">

</xml_diff>